<commit_message>
fix(workbook): a tooltip within Excel's 255 characters, one validation per column
Excel opened a rebuilt workbook with a repair: "Data validation in part
/xl/worksheets/sheet5.xml", and the ActorTypes sheet lost its list and its
tooltips. The Nature tooltip had grown to 310 characters; Excel accepts 255
for a prompt and 32 for its title, and does not truncate: it strips every
validation of the sheet. The text is shortened, and a test holds every
prompt under both limits.

The Groups sheet carried two validations on its Group column -- the
referential's list, and a bare tooltip the free-column sweep added over it.
One range, one validation: the sweep now leaves the column alone, and a test
refuses two validations on one column.

The sample workbook is regenerated with the shorter text.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSUuqeJsUPxS3rRnNRSMPV
</commit_message>
<xml_diff>
--- a/Exemples/exemple.xlsx
+++ b/Exemples/exemple.xlsx
@@ -989,7 +989,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B57"/>
+  <dimension ref="A1:B62"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="104.83203125" customWidth="1"/>
@@ -1048,7 +1048,7 @@
         <v>3. ActorTypes</v>
       </c>
       <c r="B7" t="str" s="3">
-        <v>Give each type its icon, and say whether it is Business or Technical.</v>
+        <v>Name the types your actors wear. Icon and nature are read from the referential, not typed here.</v>
       </c>
     </row>
     <row r="8">
@@ -1056,7 +1056,7 @@
         <v>4. FlowTypes</v>
       </c>
       <c r="B8" t="str" s="3">
-        <v>Keep the technologies you use, delete the rest.</v>
+        <v>Name the technologies you use. Direction, description and colour are read from the referential.</v>
       </c>
     </row>
     <row r="9">
@@ -1093,7 +1093,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str" s="2">
-        <v>THE PRINCIPLE</v>
+        <v>THE REFERENTIAL</v>
       </c>
       <c r="B13" t="str" s="2">
         <v/>
@@ -1104,7 +1104,7 @@
         <v/>
       </c>
       <c r="B14" t="str" s="3">
-        <v>An interface is PROVIDED once, by one actor, and CONSUMED by one or more others.</v>
+        <v>Actors, groups, actor types and technologies come from a shared referential: one workbook, obtained in the tool under « Repair or upgrade a workbook ».</v>
       </c>
     </row>
     <row r="15">
@@ -1112,15 +1112,15 @@
         <v/>
       </c>
       <c r="B15" t="str" s="3">
-        <v>It is described once on Interfaces, and its consumptions are detailed on an FX_&lt;provider&gt;_&lt;flow type&gt; sheet.</v>
+        <v>Drop the referential on the tool together with this workbook, or after it. This workbook carries a hidden copy of it; when that copy has drifted, the tool refreshes it and hands the updated workbook back to download.</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="str" s="3">
-        <v/>
-      </c>
-      <c r="B16" t="str" s="3">
-        <v>Two actors may publish interfaces of the same name: those are two interfaces, told apart by their provider.</v>
+      <c r="A16" t="str" s="4">
+        <v/>
+      </c>
+      <c r="B16" t="str" s="4">
+        <v>What the referential says about a name — an icon, a nature, a direction, a colour — is read from that copy, never typed here: Excel puts the formula back.</v>
       </c>
     </row>
     <row r="17">
@@ -1133,7 +1133,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str" s="2">
-        <v>THE TWO READINGS</v>
+        <v>THE PRINCIPLE</v>
       </c>
       <c r="B18" t="str" s="2">
         <v/>
@@ -1144,23 +1144,23 @@
         <v/>
       </c>
       <c r="B19" t="str" s="3">
-        <v>The same workbook is read two ways, and you fill it in only once.</v>
+        <v>An interface is PROVIDED once, by one actor, and CONSUMED by one or more others.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str" s="3">
-        <v>Architecture</v>
+        <v/>
       </c>
       <c r="B20" t="str" s="3">
-        <v>answers « what does it go through »: every hop is drawn, buses and gateways included.</v>
+        <v>It is described once on Interfaces, and its consumptions are detailed on an FX_&lt;provider&gt;_&lt;flow type&gt; sheet.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str" s="3">
-        <v>Functional</v>
+        <v/>
       </c>
       <c r="B21" t="str" s="3">
-        <v>answers « who feeds whom »: technical actors disappear, and the flows crossing them are joined end to end.</v>
+        <v>Two actors may publish interfaces of the same name: those are two interfaces, told apart by their provider.</v>
       </c>
     </row>
     <row r="22">
@@ -1168,292 +1168,332 @@
         <v/>
       </c>
       <c r="B22" t="str" s="3">
-        <v>Two columns carry the distinction, and both are optional. Nature, on ActorTypes, says which types are technical. Republished as, on the FX_ sheets, is filled on a technical actor's own consumption lines: under which of ITS interfaces that input comes back out.</v>
+        <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="str" s="3">
-        <v/>
-      </c>
-      <c r="B23" t="str" s="3">
-        <v>A bus that aggregates writes nothing special — it simply has several lines pointing at the same interface.</v>
+      <c r="A23" t="str" s="2">
+        <v>THE TWO READINGS</v>
+      </c>
+      <c r="B23" t="str" s="2">
+        <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="str" s="4">
-        <v/>
-      </c>
-      <c r="B24" t="str" s="4">
-        <v>Fill neither column and the tool never mentions the distinction.</v>
+      <c r="A24" t="str" s="3">
+        <v/>
+      </c>
+      <c r="B24" t="str" s="3">
+        <v>The same workbook is read two ways, and you fill it in only once.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str" s="3">
-        <v/>
+        <v>Architecture</v>
       </c>
       <c r="B25" t="str" s="3">
-        <v/>
+        <v>answers « what does it go through »: every hop is drawn, buses and gateways included.</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="str" s="2">
-        <v>THE SHEETS</v>
-      </c>
-      <c r="B26" t="str" s="2">
-        <v/>
+      <c r="A26" t="str" s="3">
+        <v>Functional</v>
+      </c>
+      <c r="B26" t="str" s="3">
+        <v>answers « who feeds whom »: middlewares disappear, and the flows crossing them are joined end to end.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str" s="3">
-        <v>Groups</v>
+        <v/>
       </c>
       <c r="B27" t="str" s="3">
-        <v>The perimeter is declared HERE, not on each actor: a group is Platform or External, and everything it holds follows.</v>
+        <v>Two columns carry the distinction, and both are optional. Nature, read from the referential, says what a type IS: Business, a correspondent; Middleware, plumbing that is CROSSED — a bus, a gateway; Storage, plumbing where the data STOPS — a bucket, a database, an archive. Only a middleware is folded away. Republished as, on the FX_ sheets, is filled on a middleware's own consumption lines: under which of ITS interfaces that input comes back out.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str" s="3">
-        <v>Actors</v>
+        <v/>
       </c>
       <c r="B28" t="str" s="3">
-        <v>Who exists, in which group, of which type.</v>
+        <v>A bus that aggregates writes nothing special — it simply has several lines pointing at the same interface.</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="str" s="3">
-        <v>ActorTypes</v>
-      </c>
-      <c r="B29" t="str" s="3">
-        <v>Which icon each actor type wears — and thereby the list of types that exist. Nature tells Business from Technical.</v>
+      <c r="A29" t="str" s="4">
+        <v/>
+      </c>
+      <c r="B29" t="str" s="4">
+        <v>Fill neither column and the tool never mentions the distinction.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str" s="3">
-        <v>FlowTypes</v>
+        <v/>
       </c>
       <c r="B30" t="str" s="3">
-        <v>The technologies and the direction they are drawn in.</v>
+        <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="str" s="4">
-        <v/>
-      </c>
-      <c r="B31" t="str" s="4">
-        <v>Add a Colour column to FlowTypes to pin a technology's shade, as a hex code such as #2a78d6. Without it the tool picks one from its palette; a colour too light to see is darkened on screen, and the report says so.</v>
+      <c r="A31" t="str" s="2">
+        <v>THE SHEETS</v>
+      </c>
+      <c r="B31" t="str" s="2">
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str" s="3">
-        <v>Milestones</v>
+        <v>Groups</v>
       </c>
       <c r="B32" t="str" s="3">
-        <v>The platform's timeline. Every row elsewhere says at which milestone it arrived and at which one it left.</v>
+        <v>The perimeter is declared HERE, not on each actor: a group is Platform or External, and everything it holds follows.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str" s="3">
-        <v>Interfaces</v>
+        <v>Actors</v>
       </c>
       <c r="B33" t="str" s="3">
-        <v>The catalogue: a flow, its provider, its technology, its contract.</v>
+        <v>Who exists, in which group, of which type.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str" s="3">
-        <v>FX_…</v>
+        <v>ActorTypes</v>
       </c>
       <c r="B34" t="str" s="3">
-        <v>One sheet per (provider, flow type) pair: who consumes what.</v>
+        <v>The list of types that exist here. Icon and Nature are read from the referential's copy.</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="str" s="4">
-        <v/>
-      </c>
-      <c r="B35" t="str" s="4">
-        <v>Lists and Version are hidden and filled by the tool. Right-click a tab &gt; Unhide to see them; do not edit them.</v>
+      <c r="A35" t="str" s="3">
+        <v>FlowTypes</v>
+      </c>
+      <c r="B35" t="str" s="3">
+        <v>The technologies used here. Direction, Description and Colour are read from the referential's copy.</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="str" s="3">
-        <v/>
-      </c>
-      <c r="B36" t="str" s="3">
-        <v/>
+      <c r="A36" t="str" s="4">
+        <v/>
+      </c>
+      <c r="B36" t="str" s="4">
+        <v>A technology's colour comes from the referential, as a hex code such as #2a78d6. Without one the tool picks from its palette; a colour too light to see is darkened on screen, and the report says so.</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="str" s="2">
-        <v>ENTRY RULES</v>
-      </c>
-      <c r="B37" t="str" s="2">
-        <v/>
+      <c r="A37" t="str" s="3">
+        <v>Milestones</v>
+      </c>
+      <c r="B37" t="str" s="3">
+        <v>The platform's timeline. Every row elsewhere says at which milestone it arrived and at which one it left.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str" s="3">
-        <v>Drop-down lists</v>
+        <v>Interfaces</v>
       </c>
       <c r="B38" t="str" s="3">
-        <v>Reference columns carry them and they grow by themselves: add an actor and it appears at once on Interfaces and on the FX_ sheets. Never type a name by hand — a spelling variant creates a phantom actor.</v>
+        <v>The catalogue: a flow, its provider, its technology, its contract.</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str" s="3">
-        <v>Flow name</v>
+        <v>FX_…</v>
       </c>
       <c r="B39" t="str" s="3">
-        <v>Unique for one provider, together with its version: that pair links the catalogue to the detail.</v>
+        <v>One sheet per (provider, flow type) pair: who consumes what.</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="str" s="3">
-        <v>Version</v>
-      </c>
-      <c r="B40" t="str" s="3">
-        <v>On an FX_ sheet, fill Flow name in first: the versions offered are the ones declared for that interface.</v>
+      <c r="A40" t="str" s="4">
+        <v/>
+      </c>
+      <c r="B40" t="str" s="4">
+        <v>Six sheets are hidden and filled by the tool: Lists, Version, and the referential's copy — RefActors, RefGroups, RefActorTypes, RefTechnologies. Right-click a tab &gt; Unhide to see them; do not edit them.</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str" s="3">
-        <v>Republished as</v>
+        <v/>
       </c>
       <c r="B41" t="str" s="3">
-        <v>Only on a technical actor's own consumption lines: which of its interfaces republishes this input. The drop-down offers that actor's interfaces and no others.</v>
+        <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="str" s="3">
-        <v>Decision</v>
-      </c>
-      <c r="B42" t="str" s="3">
-        <v>What has been decided for one consumption. Remove is a DEPRECATION warning, not a retirement.</v>
+      <c r="A42" t="str" s="2">
+        <v>ENTRY RULES</v>
+      </c>
+      <c r="B42" t="str" s="2">
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str" s="3">
-        <v>Retired at</v>
+        <v>Drop-down lists</v>
       </c>
       <c r="B43" t="str" s="3">
-        <v>The only column that takes a row off the diagrams. A row retired AT v3 is already gone at v3.</v>
+        <v>Reference columns carry them and they grow by themselves: add an actor and it appears at once on Interfaces and on the FX_ sheets. Never type a name by hand — a spelling variant creates a phantom actor.</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str" s="3">
-        <v>Obsolete row</v>
+        <v>Flow name</v>
       </c>
       <c r="B44" t="str" s="3">
-        <v>Do not delete it: give it a retirement milestone. Deleting it erases the history.</v>
+        <v>Unique for one provider, together with its version: that pair links the catalogue to the detail.</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str" s="3">
-        <v>Renaming an actor</v>
+        <v>Version</v>
       </c>
       <c r="B45" t="str" s="3">
-        <v>Breaks every reference to it. Find and replace across the whole workbook, or not at all.</v>
+        <v>On an FX_ sheet, fill Flow name in first: the versions offered are the ones declared for that interface.</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str" s="3">
-        <v/>
+        <v>Republished as</v>
       </c>
       <c r="B46" t="str" s="3">
-        <v/>
+        <v>Only on a middleware's own consumption lines: which of its interfaces republishes this input. The drop-down offers that actor's interfaces and no others.</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="str" s="2">
-        <v>READING AN ARROW</v>
-      </c>
-      <c r="B47" t="str" s="2">
-        <v/>
+      <c r="A47" t="str" s="3">
+        <v>Decision</v>
+      </c>
+      <c r="B47" t="str" s="3">
+        <v>What has been decided for one consumption. Remove is a DEPRECATION warning, not a retirement.</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str" s="3">
-        <v/>
+        <v>Retired at</v>
       </c>
       <c r="B48" t="str" s="3">
-        <v>Nothing to type in: two things are drawn, and both follow from the flow type.</v>
+        <v>The only column that takes a row off the diagrams. A row retired AT v3 is already gone at v3.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str" s="3">
-        <v>The line</v>
+        <v>Obsolete row</v>
       </c>
       <c r="B49" t="str" s="3">
-        <v>follows the data, always from provider to consumer, so a chain of relays reads like a pipe.</v>
+        <v>Do not delete it: give it a retirement milestone. Deleting it erases the history.</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str" s="3">
-        <v>The arrowhead</v>
+        <v>Renaming an actor</v>
       </c>
       <c r="B50" t="str" s="3">
-        <v>says who takes the initiative. A SOLID head means the provider pushes — Kafka, JMS, a file drop. An OPEN V means the consumer pulls — HTTP, SQL, LDAP — and it sits at the provider's end, pointing back at what is being queried.</v>
+        <v>Breaks every reference to it. Find and replace across the whole workbook, or not at all.</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="str" s="4">
-        <v/>
-      </c>
-      <c r="B51" t="str" s="4">
-        <v>The functional reading keeps the line and drops the nuance: a chain crosses technologies of opposite conventions, and only the data direction survives that.</v>
+      <c r="A51" t="str" s="3">
+        <v/>
+      </c>
+      <c r="B51" t="str" s="3">
+        <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="str" s="3">
-        <v/>
-      </c>
-      <c r="B52" t="str" s="3">
+      <c r="A52" t="str" s="2">
+        <v>READING AN ARROW</v>
+      </c>
+      <c r="B52" t="str" s="2">
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="str" s="2">
-        <v>MISSING FX_ SHEETS</v>
-      </c>
-      <c r="B53" t="str" s="2">
-        <v/>
+      <c r="A53" t="str" s="3">
+        <v/>
+      </c>
+      <c r="B53" t="str" s="3">
+        <v>Nothing to type in: two things are drawn, and both follow from the flow type.</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str" s="3">
-        <v/>
+        <v>The line</v>
       </c>
       <c r="B54" t="str" s="3">
+        <v>follows the data, always from provider to consumer, so a chain of relays reads like a pipe.</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str" s="3">
+        <v>The arrowhead</v>
+      </c>
+      <c r="B55" t="str" s="3">
+        <v>says who takes the initiative. A SOLID head means the provider pushes — Kafka, JMS, a file drop. An OPEN V means the consumer pulls — HTTP, SQL, LDAP — and it sits at the provider's end, pointing back at what is being queried.</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str" s="4">
+        <v/>
+      </c>
+      <c r="B56" t="str" s="4">
+        <v>The functional reading keeps the line and drops the nuance: a chain crosses technologies of opposite conventions, and only the data direction survives that.</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str" s="3">
+        <v/>
+      </c>
+      <c r="B57" t="str" s="3">
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str" s="2">
+        <v>MISSING FX_ SHEETS</v>
+      </c>
+      <c r="B58" t="str" s="2">
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str" s="3">
+        <v/>
+      </c>
+      <c r="B59" t="str" s="3">
         <v>Fill Interfaces in first: each row calls for an FX_&lt;provider&gt;_&lt;type&gt; sheet. Create it by hand, or drop this workbook on the tool and use « Repair or upgrade a workbook » — it returns the file with every expected sheet.</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="str" s="4">
-        <v/>
-      </c>
-      <c r="B55" t="str" s="4">
+    <row r="60">
+      <c r="A60" t="str" s="4">
+        <v/>
+      </c>
+      <c r="B60" t="str" s="4">
         <v>Excel caps a tab name at 31 characters and refuses \ / ? * [ ] : a long provider therefore gets a shortened tab. The tool cuts it the same way, so the two always agree, and it warns if two pairs land on the same tab.</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="str" s="3">
-        <v/>
-      </c>
-      <c r="B56" t="str" s="3">
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="str" s="4">
-        <v/>
-      </c>
-      <c r="B57" t="str" s="4">
+    <row r="61">
+      <c r="A61" t="str" s="3">
+        <v/>
+      </c>
+      <c r="B61" t="str" s="3">
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str" s="4">
+        <v/>
+      </c>
+      <c r="B62" t="str" s="4">
         <v>The visualisation tool only READS this workbook: it never modifies it.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B62"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1593,7 +1633,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Decision" prompt="What has been decided for this consumption. Remove is a deprecation warning, not a retirement: retirement is the Retired at column." sqref="F2:F1000">
       <formula1>L_Decision</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a technical actor: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a middleware: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
       <formula1>OFFSET(Lists!$Q$2,MATCH($C2,Lists!$P$2:$P$1018,0)-1,0,MAX(1,COUNTIF(Lists!$P$2:$P$1018,$C2)),1)</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Introduced at" prompt="A milestone from the Milestones sheet, the one this line appears at. Leave empty if it has always been there." sqref="I2:I1000">
@@ -1845,7 +1885,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Decision" prompt="What has been decided for this consumption. Remove is a deprecation warning, not a retirement: retirement is the Retired at column." sqref="F2:F1000">
       <formula1>L_Decision</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a technical actor: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a middleware: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
       <formula1>OFFSET(Lists!$Q$2,MATCH($C2,Lists!$P$2:$P$1018,0)-1,0,MAX(1,COUNTIF(Lists!$P$2:$P$1018,$C2)),1)</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Introduced at" prompt="A milestone from the Milestones sheet, the one this line appears at. Leave empty if it has always been there." sqref="I2:I1000">
@@ -1969,7 +2009,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Decision" prompt="What has been decided for this consumption. Remove is a deprecation warning, not a retirement: retirement is the Retired at column." sqref="F2:F1000">
       <formula1>L_Decision</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a technical actor: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a middleware: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
       <formula1>OFFSET(Lists!$Q$2,MATCH($C2,Lists!$P$2:$P$1018,0)-1,0,MAX(1,COUNTIF(Lists!$P$2:$P$1018,$C2)),1)</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Introduced at" prompt="A milestone from the Milestones sheet, the one this line appears at. Leave empty if it has always been there." sqref="I2:I1000">
@@ -2093,7 +2133,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Decision" prompt="What has been decided for this consumption. Remove is a deprecation warning, not a retirement: retirement is the Retired at column." sqref="F2:F1000">
       <formula1>L_Decision</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a technical actor: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a middleware: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
       <formula1>OFFSET(Lists!$Q$2,MATCH($C2,Lists!$P$2:$P$1018,0)-1,0,MAX(1,COUNTIF(Lists!$P$2:$P$1018,$C2)),1)</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Introduced at" prompt="A milestone from the Milestones sheet, the one this line appears at. Leave empty if it has always been there." sqref="I2:I1000">
@@ -2217,7 +2257,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Decision" prompt="What has been decided for this consumption. Remove is a deprecation warning, not a retirement: retirement is the Retired at column." sqref="F2:F1000">
       <formula1>L_Decision</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a technical actor: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a middleware: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
       <formula1>OFFSET(Lists!$Q$2,MATCH($C2,Lists!$P$2:$P$1018,0)-1,0,MAX(1,COUNTIF(Lists!$P$2:$P$1018,$C2)),1)</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Introduced at" prompt="A milestone from the Milestones sheet, the one this line appears at. Leave empty if it has always been there." sqref="I2:I1000">
@@ -2405,7 +2445,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Decision" prompt="What has been decided for this consumption. Remove is a deprecation warning, not a retirement: retirement is the Retired at column." sqref="F2:F1000">
       <formula1>L_Decision</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a technical actor: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a middleware: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
       <formula1>OFFSET(Lists!$Q$2,MATCH($C2,Lists!$P$2:$P$1018,0)-1,0,MAX(1,COUNTIF(Lists!$P$2:$P$1018,$C2)),1)</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Introduced at" prompt="A milestone from the Milestones sheet, the one this line appears at. Leave empty if it has always been there." sqref="I2:I1000">
@@ -2529,7 +2569,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Decision" prompt="What has been decided for this consumption. Remove is a deprecation warning, not a retirement: retirement is the Retired at column." sqref="F2:F1000">
       <formula1>L_Decision</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a technical actor: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a middleware: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
       <formula1>OFFSET(Lists!$Q$2,MATCH($C2,Lists!$P$2:$P$1018,0)-1,0,MAX(1,COUNTIF(Lists!$P$2:$P$1018,$C2)),1)</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Introduced at" prompt="A milestone from the Milestones sheet, the one this line appears at. Leave empty if it has always been there." sqref="I2:I1000">
@@ -2653,7 +2693,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Decision" prompt="What has been decided for this consumption. Remove is a deprecation warning, not a retirement: retirement is the Retired at column." sqref="F2:F1000">
       <formula1>L_Decision</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a technical actor: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a middleware: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
       <formula1>OFFSET(Lists!$Q$2,MATCH($C2,Lists!$P$2:$P$1018,0)-1,0,MAX(1,COUNTIF(Lists!$P$2:$P$1018,$C2)),1)</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Introduced at" prompt="A milestone from the Milestones sheet, the one this line appears at. Leave empty if it has always been there." sqref="I2:I1000">
@@ -2777,7 +2817,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Decision" prompt="What has been decided for this consumption. Remove is a deprecation warning, not a retirement: retirement is the Retired at column." sqref="F2:F1000">
       <formula1>L_Decision</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a technical actor: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a middleware: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
       <formula1>OFFSET(Lists!$Q$2,MATCH($C2,Lists!$P$2:$P$1018,0)-1,0,MAX(1,COUNTIF(Lists!$P$2:$P$1018,$C2)),1)</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Introduced at" prompt="A milestone from the Milestones sheet, the one this line appears at. Leave empty if it has always been there." sqref="I2:I1000">
@@ -2933,7 +2973,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Decision" prompt="What has been decided for this consumption. Remove is a deprecation warning, not a retirement: retirement is the Retired at column." sqref="F2:F1000">
       <formula1>L_Decision</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a technical actor: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a middleware: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
       <formula1>OFFSET(Lists!$Q$2,MATCH($C2,Lists!$P$2:$P$1018,0)-1,0,MAX(1,COUNTIF(Lists!$P$2:$P$1018,$C2)),1)</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Introduced at" prompt="A milestone from the Milestones sheet, the one this line appears at. Leave empty if it has always been there." sqref="I2:I1000">
@@ -3418,7 +3458,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Group" prompt="The group this component belongs to. The group carries the perimeter — Platform or External — so everything it holds follows." sqref="B2:B1000">
       <formula1>L_Groupe</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Actor type" prompt="Declared on the ActorTypes sheet, which also gives it its icon and says whether it is business or technical." sqref="C2:C1000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Actor type" prompt="Declared on the ActorTypes sheet; its icon and its nature — Business, Middleware or Storage — are read from the referential." sqref="C2:C1000">
       <formula1>L_TypeActeur</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Introduced at" prompt="A milestone from the Milestones sheet, the one this line appears at. Leave empty if it has always been there." sqref="G2:G1000">
@@ -3543,7 +3583,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Decision" prompt="What has been decided for this consumption. Remove is a deprecation warning, not a retirement: retirement is the Retired at column." sqref="F2:F1000">
       <formula1>L_Decision</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a technical actor: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a middleware: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
       <formula1>OFFSET(Lists!$Q$2,MATCH($C2,Lists!$P$2:$P$1018,0)-1,0,MAX(1,COUNTIF(Lists!$P$2:$P$1018,$C2)),1)</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Introduced at" prompt="A milestone from the Milestones sheet, the one this line appears at. Leave empty if it has always been there." sqref="I2:I1000">
@@ -3667,7 +3707,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Decision" prompt="What has been decided for this consumption. Remove is a deprecation warning, not a retirement: retirement is the Retired at column." sqref="F2:F1000">
       <formula1>L_Decision</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a technical actor: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a middleware: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
       <formula1>OFFSET(Lists!$Q$2,MATCH($C2,Lists!$P$2:$P$1018,0)-1,0,MAX(1,COUNTIF(Lists!$P$2:$P$1018,$C2)),1)</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Introduced at" prompt="A milestone from the Milestones sheet, the one this line appears at. Leave empty if it has always been there." sqref="I2:I1000">
@@ -3791,7 +3831,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Decision" prompt="What has been decided for this consumption. Remove is a deprecation warning, not a retirement: retirement is the Retired at column." sqref="F2:F1000">
       <formula1>L_Decision</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a technical actor: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a middleware: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
       <formula1>OFFSET(Lists!$Q$2,MATCH($C2,Lists!$P$2:$P$1018,0)-1,0,MAX(1,COUNTIF(Lists!$P$2:$P$1018,$C2)),1)</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Introduced at" prompt="A milestone from the Milestones sheet, the one this line appears at. Leave empty if it has always been there." sqref="I2:I1000">
@@ -6388,14 +6428,13 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0" promptTitle="Group" prompt="The group this component belongs to. The group carries the perimeter — Platform or External — so everything it holds follows." sqref="A2:A1000">
       <formula1>L_RefGroupe</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Perimeter" prompt="Platform for what the team owns, External for the rest. This is what decides how the group is drawn." sqref="B2:B1000">
       <formula1>L_Perimetre</formula1>
     </dataValidation>
-    <dataValidation type="none" allowBlank="1" showInputMessage="1" showErrorMessage="0" promptTitle="Group" prompt="The group this component belongs to. The group carries the perimeter — Platform or External — so everything it holds follows." sqref="A2:A1000"/>
   </dataValidations>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
@@ -6629,11 +6668,11 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0" promptTitle="Actor type" prompt="Declared on the ActorTypes sheet, which also gives it its icon and says whether it is business or technical." sqref="A2:A1000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="0" promptTitle="Actor type" prompt="Declared on the ActorTypes sheet; its icon and its nature — Business, Middleware or Storage — are read from the referential." sqref="A2:A1000">
       <formula1>L_RefTypeActeur</formula1>
     </dataValidation>
     <dataValidation type="none" allowBlank="1" showInputMessage="1" showErrorMessage="0" promptTitle="Icon" prompt="Read from the referential for this type. Not entered here: Excel puts the formula back. Change it in the referential, then drop the referential on the tool with this workbook." sqref="B2:B1000"/>
-    <dataValidation type="none" allowBlank="1" showInputMessage="1" showErrorMessage="0" promptTitle="Nature" prompt="Read from the referential. A technical type is traversed in the functional reading: its actors do not appear, and the flows through them are joined end to end. Change it in the referential, then drop the referential on the tool with this workbook." sqref="C2:C1000"/>
+    <dataValidation type="none" allowBlank="1" showInputMessage="1" showErrorMessage="0" promptTitle="Nature" prompt="Read from the referential: Business, Middleware or Storage. A middleware is crossed in the functional reading, its flows joined end to end; a storage is where the data stops. Change it in the referential, then drop that on the tool with this workbook." sqref="C2:C1000"/>
   </dataValidations>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
@@ -7872,7 +7911,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Decision" prompt="What has been decided for this consumption. Remove is a deprecation warning, not a retirement: retirement is the Retired at column." sqref="F2:F1000">
       <formula1>L_Decision</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a technical actor: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a middleware: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
       <formula1>OFFSET(Lists!$Q$2,MATCH($C2,Lists!$P$2:$P$1018,0)-1,0,MAX(1,COUNTIF(Lists!$P$2:$P$1018,$C2)),1)</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Introduced at" prompt="A milestone from the Milestones sheet, the one this line appears at. Leave empty if it has always been there." sqref="I2:I1000">
@@ -8060,7 +8099,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Decision" prompt="What has been decided for this consumption. Remove is a deprecation warning, not a retirement: retirement is the Retired at column." sqref="F2:F1000">
       <formula1>L_Decision</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a technical actor: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Republished as" prompt="Fill in only when the consumer is a middleware: which of ITS OWN interfaces republishes this flow. Several lines pointing at the same interface is how a bus aggregates." sqref="H2:H1000">
       <formula1>OFFSET(Lists!$Q$2,MATCH($C2,Lists!$P$2:$P$1018,0)-1,0,MAX(1,COUNTIF(Lists!$P$2:$P$1018,$C2)),1)</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Introduced at" prompt="A milestone from the Milestones sheet, the one this line appears at. Leave empty if it has always been there." sqref="I2:I1000">

</xml_diff>